<commit_message>
feat(receivables): add interactive inline editing and modal support
- Enable inline editing for tax rates, due dates, paid dates, and received amounts

- Add full edit and create modals for receivables tracker

- Enhance fullscreen viewport mode and horizontal scrolling navigation
</commit_message>
<xml_diff>
--- a/Ho So Du An/Yeu Cau Thanh Toan/HM21102026-001_Phiếu_Yêu_Cầu_Thanh_Toán_CÔNG TY CỔ PHẦN CX TECHNOLOGY _HMV151020250001.xlsx
+++ b/Ho So Du An/Yeu Cau Thanh Toan/HM21102026-001_Phiếu_Yêu_Cầu_Thanh_Toán_CÔNG TY CỔ PHẦN CX TECHNOLOGY _HMV151020250001.xlsx
@@ -1543,9 +1543,9 @@
       <c r="C11" s="72" t="inlineStr">
         <is>
           <t>Căn cứ hợp đồng số : HMV151020250001
-RFID Hardware &amp; Custom Software ERP
+RFID 硬體 (RFID Hardware) – Phần mềm tùy chỉnh chức năng hệ thống RFID
 根据合同编号：HMV151020250001
-RFID硬體與系統客製化軟體</t>
+RFID硬體（RFID Hardware）－RFID系統客製化軟體</t>
         </is>
       </c>
       <c r="K11" s="83" t="n"/>
@@ -1640,7 +1640,7 @@
       </c>
       <c r="B15" s="39" t="inlineStr">
         <is>
-          <t>驗收合格尾款：20%
+          <t>驗收合格尾款：20% (Thanh toán đợt Giai đoạn 3 - 20% Nghiệm thu đạt tiêu chuẩn)
 合約：HMV151020250001</t>
         </is>
       </c>
@@ -1813,7 +1813,12 @@
       <c r="A23" s="38" t="n"/>
       <c r="B23" s="97" t="inlineStr">
         <is>
-          <t xml:space="preserve">備註：1. 40% = 93.600.000 VND; 2. 40% = 93.600.000 VND; 3. 20% = 46.800.000 VND.
+          <t xml:space="preserve">備註：1. Sau khi ký kết hợp đồng: thanh toán 40% giá trị hợp đồng = 93.600.000 VNĐ.
+1. 簽約完成時：支付合約金額40%＝93,600,000越盾。
+2. Sau khi triển khai sản phẩm đưa vào sử dụng: thanh toán 40% giá trị hợp đồng = 93.600.000 VNĐ.
+2. 產品安裝後：支付合約金額40%＝93,600,000越盾。
+3. Khi nghiệm thu đạt tiêu chuẩn: thanh toán 20% còn lại = 46.800.000 VNĐ.
+3. 驗收合格時：支付尾款20%＝46,800,000越盾。
 **以上價格不包含VAT增值稅，稅率依發票開立時的稅率為準。Giá nêu trên chưa bao gồm thuế GTGT (VAT). Thuế suất áp dụng theo mức thuế suất tại thời điểm xuất hóa đơn.
 </t>
         </is>

</xml_diff>